<commit_message>
fix(verfal): Tambahkan kolom NO.KK pada Lamp.IIIA Template Verfal dan perbarui parser upload
</commit_message>
<xml_diff>
--- a/TEMPLATE_VERFAL.xlsx
+++ b/TEMPLATE_VERFAL.xlsx
@@ -2,22 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lamp.IIA" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lamp.IIIA" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,20 +27,27 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <family val="2"/>
+      <name val="Bookman Old Style"/>
       <b val="1"/>
-      <sz val="11"/>
+      <sz val="14"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <family val="2"/>
+      <name val="Bookman Old Style"/>
       <b val="1"/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="11"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Bookman Old Style"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Bookman Old Style"/>
+      <b val="1"/>
+      <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -48,24 +56,30 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF4472C4"/>
-        <bgColor rgb="FF4472C4"/>
+        <fgColor rgb="00305496"/>
+        <bgColor rgb="00305496"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC00000"/>
-        <bgColor rgb="FFC00000"/>
+        <fgColor rgb="00ED7D31"/>
+        <bgColor rgb="00ED7D31"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF548235"/>
-        <bgColor rgb="FF548235"/>
+        <fgColor rgb="00C00000"/>
+        <bgColor rgb="00C00000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00375623"/>
+        <bgColor rgb="00375623"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -73,34 +87,56 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -461,131 +497,224 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A3:M9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <dimension ref="A3:M10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" style="7" min="1" max="1"/>
-    <col width="25" customWidth="1" style="7" min="2" max="2"/>
-    <col width="14" customWidth="1" style="7" min="3" max="3"/>
-    <col width="18" customWidth="1" style="7" min="4" max="4"/>
-    <col width="22.21875" customWidth="1" style="7" min="5" max="5"/>
-    <col width="25" customWidth="1" style="7" min="6" max="6"/>
-    <col width="18" customWidth="1" style="7" min="7" max="7"/>
-    <col width="13" customWidth="1" style="7" min="8" max="8"/>
-    <col width="23.6640625" customWidth="1" style="7" min="9" max="9"/>
-    <col width="14" customWidth="1" style="7" min="10" max="10"/>
-    <col width="10" customWidth="1" style="7" min="11" max="11"/>
-    <col width="14" customWidth="1" style="7" min="12" max="12"/>
-    <col width="20" customWidth="1" style="7" min="13" max="13"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
-    <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+    <row r="1" ht="20" customHeight="1"/>
+    <row r="2" ht="20" customHeight="1"/>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>DAFTAR HASIL VERIFIKASI FAKTUAL CALON PENERIMA BANTUAN</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>BEDAH RUMAH TAHUN [Tahun Anggaran]</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>PROVINSI [Provinsi Aktif]</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="K8" s="4" t="inlineStr">
-        <is>
-          <t>INSTRUKSI VERIFIKASI</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="28.8" customHeight="1" s="7">
-      <c r="A9" s="4" t="inlineStr">
+    <row r="6" ht="20" customHeight="1"/>
+    <row r="7" ht="20" customHeight="1"/>
+    <row r="8" ht="24" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>NO. URUT</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>NAMA</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>JENIS
 KELAMIN (L/P)</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>NO.KTP</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>NO.KK</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>ALAMAT TEMPAT
 TINGGAL</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>DESA / KELURAHAN</t>
         </is>
       </c>
-      <c r="H9" s="4" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>KECAMATAN</t>
         </is>
       </c>
-      <c r="I9" s="4" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>KABUPATEN / KOTA</t>
         </is>
       </c>
-      <c r="J9" s="4" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>LOLOS/TIDAK LOLOS</t>
         </is>
       </c>
-      <c r="K9" s="4" t="inlineStr">
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>INSTRUKSI VERIFIKASI</t>
+        </is>
+      </c>
+      <c r="L8" s="3" t="n"/>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>KETERANGAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="32" customHeight="1">
+      <c r="A9" s="2" t="n"/>
+      <c r="B9" s="2" t="n"/>
+      <c r="C9" s="2" t="n"/>
+      <c r="D9" s="2" t="n"/>
+      <c r="E9" s="2" t="n"/>
+      <c r="F9" s="2" t="n"/>
+      <c r="G9" s="2" t="n"/>
+      <c r="H9" s="2" t="n"/>
+      <c r="I9" s="2" t="n"/>
+      <c r="J9" s="2" t="n"/>
+      <c r="K9" s="3" t="inlineStr">
         <is>
           <t>TAHAP</t>
         </is>
       </c>
-      <c r="L9" s="4" t="inlineStr">
+      <c r="L9" s="3" t="inlineStr">
         <is>
           <t>TANGGAL</t>
         </is>
       </c>
-      <c r="M9" s="4" t="inlineStr">
-        <is>
-          <t>KETERANGAN</t>
+      <c r="M9" s="2" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>CONTOH NAMA LOLOS</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>'7301010101010001</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>'7301010101010002</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>DUSUN MAJU</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>DESA A</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>KECAMATAN B</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>KABUPATEN C</t>
+        </is>
+      </c>
+      <c r="J10" s="4" t="inlineStr">
+        <is>
+          <t>LOLOS</t>
+        </is>
+      </c>
+      <c r="K10" s="4" t="inlineStr">
+        <is>
+          <t>Tahap 1</t>
+        </is>
+      </c>
+      <c r="L10" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="M10" s="5" t="inlineStr">
+        <is>
+          <t>Memenuhi Syarat</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="15">
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="A5:M5"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="E8:E9"/>
+    <mergeCell ref="K8:L8"/>
+    <mergeCell ref="F8:F9"/>
+    <mergeCell ref="G8:G9"/>
+    <mergeCell ref="H8:H9"/>
+    <mergeCell ref="I8:I9"/>
+    <mergeCell ref="J8:J9"/>
+    <mergeCell ref="M8:M9"/>
     <mergeCell ref="A4:M4"/>
-    <mergeCell ref="K8:L8"/>
+    <mergeCell ref="D8:D9"/>
     <mergeCell ref="A3:M3"/>
-    <mergeCell ref="A5:M5"/>
+    <mergeCell ref="B8:B9"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -593,204 +722,407 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <dimension ref="A3:V22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" style="7" min="1" max="1"/>
-    <col width="25" customWidth="1" style="7" min="2" max="2"/>
-    <col width="14" customWidth="1" style="7" min="3" max="3"/>
-    <col width="18" customWidth="1" style="7" min="4" max="4"/>
-    <col width="25" customWidth="1" style="7" min="5" max="5"/>
-    <col width="18" customWidth="1" style="7" min="6" max="6"/>
-    <col width="15" customWidth="1" style="7" min="7" max="8"/>
-    <col width="16" customWidth="1" style="7" min="9" max="9"/>
-    <col width="8" customWidth="1" style="7" min="10" max="10"/>
-    <col width="25" customWidth="1" style="7" min="11" max="11"/>
-    <col width="14" customWidth="1" style="7" min="12" max="12"/>
-    <col width="18" customWidth="1" style="7" min="13" max="13"/>
-    <col width="20" customWidth="1" style="7" min="14" max="14"/>
-    <col width="18" customWidth="1" style="7" min="15" max="15"/>
-    <col width="15" customWidth="1" style="7" min="16" max="17"/>
-    <col width="10" customWidth="1" style="7" min="18" max="18"/>
-    <col width="14" customWidth="1" style="7" min="19" max="19"/>
-    <col width="20" customWidth="1" style="7" min="20" max="20"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="28" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
+    <col width="24" customWidth="1" min="15" max="15"/>
+    <col width="28" customWidth="1" min="16" max="16"/>
+    <col width="22" customWidth="1" min="17" max="17"/>
+    <col width="22" customWidth="1" min="18" max="18"/>
+    <col width="22" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="24" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
-    <row r="1"/>
-    <row r="2"/>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>DAFTAR CALON PENGGANTI PENERIMA BANTUAN</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>BEDAH RUMAH TAHUN [Tahun Anggaran]</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>PROVINSI [Provinsi Aktif]</t>
         </is>
       </c>
     </row>
-    <row r="6"/>
-    <row r="7">
-      <c r="B7" s="2" t="inlineStr">
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>NO.</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>TIDAK LOLOS</t>
         </is>
       </c>
-      <c r="J7" s="8" t="inlineStr">
-        <is>
-          <t>SEMUA</t>
-        </is>
-      </c>
-      <c r="K7" s="8" t="n"/>
-      <c r="L7" s="8" t="n"/>
-      <c r="M7" s="8" t="n"/>
-      <c r="N7" s="8" t="n"/>
-      <c r="O7" s="8" t="n"/>
-      <c r="P7" s="8" t="n"/>
-      <c r="Q7" s="8" t="n"/>
-      <c r="R7" s="8" t="n"/>
-      <c r="S7" s="4" t="inlineStr">
+      <c r="C7" s="7" t="n"/>
+      <c r="D7" s="7" t="n"/>
+      <c r="E7" s="7" t="n"/>
+      <c r="F7" s="7" t="n"/>
+      <c r="G7" s="7" t="n"/>
+      <c r="H7" s="7" t="n"/>
+      <c r="I7" s="7" t="n"/>
+      <c r="J7" s="7" t="n"/>
+      <c r="K7" s="8" t="inlineStr">
+        <is>
+          <t>PENGGANTI</t>
+        </is>
+      </c>
+      <c r="L7" s="9" t="n"/>
+      <c r="M7" s="9" t="n"/>
+      <c r="N7" s="9" t="n"/>
+      <c r="O7" s="9" t="n"/>
+      <c r="P7" s="9" t="n"/>
+      <c r="Q7" s="9" t="n"/>
+      <c r="R7" s="9" t="n"/>
+      <c r="S7" s="9" t="n"/>
+      <c r="T7" s="3" t="inlineStr">
         <is>
           <t>INSTRUKSI VERIFIKASI</t>
         </is>
       </c>
-    </row>
-    <row r="8" ht="28.8" customHeight="1" s="7">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>NO.</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="U7" s="10" t="n"/>
+      <c r="V7" s="2" t="inlineStr">
+        <is>
+          <t>KETERANGAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="34" customHeight="1">
+      <c r="A8" s="11" t="n"/>
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>NAMA</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>JENIS KELAMIN
 (L/P)</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>NO.KTP</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>NO.KK</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>ALAMAT TEMPAT
 TINGGAL</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>DESA / KELURAHAN</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>KECAMATAN</t>
         </is>
       </c>
-      <c r="H8" s="4" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>KABUPATEN</t>
         </is>
       </c>
-      <c r="I8" s="4" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>ALASAN TIDAK
 LOLOS *)</t>
         </is>
       </c>
-      <c r="J8" s="4" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>BNBA</t>
         </is>
       </c>
-      <c r="K8" s="4" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>NAMA
 (PENGGANTI)</t>
         </is>
       </c>
-      <c r="L8" s="4" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>JENIS KELAMIN
 (L/P)</t>
         </is>
       </c>
-      <c r="M8" s="4" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>NO.KTP
 (PENGGANTI)</t>
         </is>
       </c>
-      <c r="N8" s="4" t="inlineStr">
+      <c r="O8" s="2" t="inlineStr">
         <is>
           <t>NO.KK
 (PENGGANTI)</t>
         </is>
       </c>
-      <c r="O8" s="4" t="inlineStr">
+      <c r="P8" s="2" t="inlineStr">
         <is>
           <t>ALAMAT TEMPAT
 TINGGAL</t>
         </is>
       </c>
-      <c r="P8" s="4" t="inlineStr">
+      <c r="Q8" s="2" t="inlineStr">
         <is>
           <t>DESA / KELURAHAN</t>
         </is>
       </c>
-      <c r="Q8" s="4" t="inlineStr">
+      <c r="R8" s="2" t="inlineStr">
         <is>
           <t>KECAMATAN</t>
         </is>
       </c>
-      <c r="R8" s="4" t="inlineStr">
+      <c r="S8" s="2" t="inlineStr">
         <is>
           <t>KABUPATEN</t>
         </is>
       </c>
-      <c r="S8" s="4" t="inlineStr">
+      <c r="T8" s="3" t="inlineStr">
         <is>
           <t>TAHAP</t>
         </is>
       </c>
-      <c r="T8" s="4" t="inlineStr">
+      <c r="U8" s="3" t="inlineStr">
         <is>
           <t>TANGGAL</t>
         </is>
       </c>
-      <c r="U8" s="4" t="inlineStr">
-        <is>
-          <t>KETERANGAN</t>
+      <c r="V8" s="11" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>CONTOH NAMA TIDAK LOLOS</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>'7301010101010003</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>'7301010101010004</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>DUSUN LAMA</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>DESA A</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>KECAMATAN B</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>KABUPATEN C</t>
+        </is>
+      </c>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K9" s="4" t="inlineStr"/>
+      <c r="L9" s="5" t="inlineStr">
+        <is>
+          <t>CONTOH NAMA PENGGANTI</t>
+        </is>
+      </c>
+      <c r="M9" s="4" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="N9" s="4" t="inlineStr">
+        <is>
+          <t>'7301010101010005</t>
+        </is>
+      </c>
+      <c r="O9" s="4" t="inlineStr">
+        <is>
+          <t>'7301010101010006</t>
+        </is>
+      </c>
+      <c r="P9" s="5" t="inlineStr">
+        <is>
+          <t>DUSUN BARU</t>
+        </is>
+      </c>
+      <c r="Q9" s="5" t="inlineStr">
+        <is>
+          <t>DESA A</t>
+        </is>
+      </c>
+      <c r="R9" s="5" t="inlineStr">
+        <is>
+          <t>KECAMATAN B</t>
+        </is>
+      </c>
+      <c r="S9" s="5" t="inlineStr">
+        <is>
+          <t>KABUPATEN C</t>
+        </is>
+      </c>
+      <c r="T9" s="4" t="inlineStr">
+        <is>
+          <t>Tahap 1</t>
+        </is>
+      </c>
+      <c r="U9" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="V9" s="5" t="inlineStr">
+        <is>
+          <t>Pengganti</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>Catatan:</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>*) Alasan Tidak Lolos, diisi dengan angka (1-8) sebagai berikut:</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>1. Belum memiliki KK sendiri;</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="13" t="inlineStr">
+        <is>
+          <t>2. Tanah bersengketa;</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>3. Rumah dalam kondisi layak;</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t>4. Memiliki rumah lebih dari 1;</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="13" t="inlineStr">
+        <is>
+          <t>5. Pernah memperoleh bantuan dari APBN/APBD/CSR/anggaran lainnya;</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="13" t="inlineStr">
+        <is>
+          <t>6. Penghasilan lebih dari UMP;</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>7. Memilih untuk dibantu dengan sumber anggaran lain;</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="13" t="inlineStr">
+        <is>
+          <t>8. Menghuni kurang dari 3 tahun;</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="13" t="inlineStr">
+        <is>
+          <t>9. Lainnya (diisi pada kolom keterangan);</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="A4:U4"/>
-    <mergeCell ref="B7:I7"/>
-    <mergeCell ref="J7:R7"/>
-    <mergeCell ref="S7:T7"/>
-    <mergeCell ref="A5:U5"/>
-    <mergeCell ref="A3:U3"/>
+  <mergeCells count="8">
+    <mergeCell ref="B7:J7"/>
+    <mergeCell ref="T7:U7"/>
+    <mergeCell ref="A5:V5"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="V7:V8"/>
+    <mergeCell ref="A3:V3"/>
+    <mergeCell ref="A4:V4"/>
+    <mergeCell ref="K7:S7"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>